<commit_message>
v2.0.4: one-click ffmpeg download (gyan.dev, SHA-256 verified, GPL v3 notice), winget --source fix, updated locationGPS.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/locationGPS.xlsx
+++ b/locationGPS.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\skypr\Downloads\gpx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\HikeReel_v2.0.3_Windows\HikeReel_v2.0.3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A0BAB1C-3A7F-4494-B817-24300DE5DB3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB644E5B-3953-4561-A858-5EC667C7BFD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="地標總庫" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="78">
   <si>
     <t>名稱</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t>選填</t>
-  </si>
-  <si>
-    <t>停車場</t>
   </si>
   <si>
     <t>Tre Cime</t>
@@ -142,11 +139,6 @@
     <t>--radius 1.0</t>
   </si>
   <si>
-    <t>教堂
-Cappella degli Alpini</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>46.63692277593782, 12.31052613663016</t>
   </si>
   <si>
@@ -251,11 +243,6 @@
   <si>
     <t>纜車
 Funicolare Resciesa</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
-    <t>三尖峰側面
-Forcella Lavaredo</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
@@ -298,6 +285,25 @@
   </si>
   <si>
     <t>46.623709116741615, 11.775439716418271</t>
+  </si>
+  <si>
+    <t>阿爾卑斯小教堂
+Cappella degli Alpini</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>拉瓦雷多埡口
+Forcella Lavaredo</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>三尖峰停車場</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>教堂
+Cappella Lago di Braies</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -747,15 +753,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="19.6171875" customWidth="1"/>
+    <col min="3" max="3" width="19.59765625" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -769,7 +775,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -783,266 +789,266 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5"/>
+    </row>
+    <row r="4" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5"/>
+    </row>
+    <row r="6" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="5"/>
-    </row>
-    <row r="4" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A4" s="5" t="s">
+      <c r="B10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="4"/>
+    </row>
+    <row r="11" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="4"/>
+    </row>
+    <row r="12" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" s="4"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="4"/>
+    </row>
+    <row r="14" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A14" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="4"/>
+    </row>
+    <row r="15" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="29" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A19" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A5" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="5"/>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A7" s="5" t="s">
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A20" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="B20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A21" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B21" t="s">
+        <v>62</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="B22" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A8" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D9" s="5"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.7">
-      <c r="A10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="4"/>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A11" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D11" s="4"/>
-    </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A12" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.7">
-      <c r="A13" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A14" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D14" s="4"/>
-    </row>
-    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A15" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="B15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.7">
-      <c r="A16" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A17" s="11" t="s">
+    </row>
+    <row r="23" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A23" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="B23" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="29" x14ac:dyDescent="0.3">
+      <c r="A24" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B17" t="s">
-        <v>57</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="45" x14ac:dyDescent="0.7">
-      <c r="A18" s="3" t="s">
+      <c r="B24" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" t="s">
         <v>70</v>
-      </c>
-      <c r="B18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A19" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A20" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A21" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.7">
-      <c r="A22" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B22" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A23" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="B23" t="s">
-        <v>72</v>
-      </c>
-      <c r="C23" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.7">
-      <c r="A24" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="B24" t="s">
-        <v>76</v>
-      </c>
-      <c r="C24" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1054,52 +1060,52 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>0</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.7">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>1</v>
       </c>
       <c r="B5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="B6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>2</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -1107,53 +1113,53 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.7">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A11" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A12" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A13" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A15" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>31</v>
       </c>
-      <c r="B16" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A17" t="s">
+      <c r="B17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.7">
-      <c r="A18" t="s">
+      <c r="B18" t="s">
         <v>35</v>
-      </c>
-      <c r="B18" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>